<commit_message>
Add Due Date field to bulk and manual reminder/receipt emails
New "Due Date" column in the bulk email template (required, next to
Billing Date) and a matching "Next Due Date" field on the manual Send
Email form (optional there, since a one-off send doesn't always have
one). Both flow into a new "Next due date:" row in the receipt and
reminder templates.

Cancellation date stays auto-computed as billing date + 1 day, not a
spreadsheet column — unchanged from before, just re-verified end to
end after the Due Date row was added alongside it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/bulk-email-template.xlsx
+++ b/public/templates/bulk-email-template.xlsx
@@ -27,12 +27,11 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
     </font>
     <font>
       <i val="1"/>
-      <color rgb="009AA0A6"/>
+      <color rgb="FF9AA0A6"/>
     </font>
   </fonts>
   <fills count="4">
@@ -44,12 +43,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0000254A"/>
+        <fgColor rgb="FF00254A"/>
+        <bgColor rgb="FF00254A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002CA01C"/>
+        <fgColor rgb="FF2CA01C"/>
+        <bgColor rgb="FF2CA01C"/>
       </patternFill>
     </fill>
   </fills>
@@ -65,16 +66,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -154,19 +154,19 @@
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>QB Enterprise</author>
+    <author>QuickBooks Enterprise</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
         <t>Optional
-Shown as 'Company name:' in the email. Falls back to the customer's name if blank.</t>
+Shown as ‘Company name:’ in the email. Falls back to the customer’s name if blank.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
         <t>Optional
-Used in the greeting: 'Hi {First Name},'</t>
+Used in the greeting: ‘Hi {First Name},’</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
@@ -190,22 +190,28 @@
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
         <t>REQUIRED
-REQUIRED. Shown as 'Affected subscriptions:', e.g. QuickBooks Enterprise Silver Edition</t>
+REQUIRED. Format YYYY-MM-DD, e.g. 2026-09-14. Shown in the email as ‘Next due date:’ — when this subscription is next charged.</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
       <text>
+        <t>REQUIRED
+REQUIRED. Shown as ‘Affected subscriptions:’, e.g. QuickBooks Enterprise Silver Edition</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
         <t>Optional
-Shown as 'Payment method:', e.g. VISA ending in 1234. Defaults to 'the payment method on file'.</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
+Shown as ‘Payment method:’, e.g. VISA ending in 1234. Defaults to ‘the payment method on file’.</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
       <text>
         <t>Optional
 Reference only — not shown in reminder emails.</t>
       </text>
     </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
+    <comment ref="K1" authorId="0" shapeId="0">
       <text>
         <t>Optional
 Reference only — not shown in reminder emails.</t>
@@ -504,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -513,13 +519,14 @@
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Company Name</t>
@@ -552,20 +559,25 @@
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Current Payment method</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>License Number</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>CAN</t>
         </is>
@@ -592,7 +604,7 @@
           <t>jane@acme.com</t>
         </is>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="E2" s="3" t="n">
         <v>349.89</v>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -602,20 +614,25 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
           <t>QuickBooks Enterprise Silver Edition</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>VISA ending in 1234</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>1234-5678-9012-345</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>CAN-00417</t>
         </is>

</xml_diff>

<commit_message>
Remove Billing Date, rename Next due date to Due date
Billing Date was a redundant third date on top of Due Date and
Cancellation Date, and easy to fill in wrong. Reminder emails now
show only Due date and Cancellation date (cancellation = due date +
1 day, same relationship as before, just anchored on the due date
instead). The Excel template drops the column entirely; old sheets
with a "Billing Date" header still map into Due Date so an existing
file isn't broken by the rename. The manual Send Email form drops
its Billing Date input and makes Due Date required, matching bulk.

"Next due date:" becomes "Due date:" in both templates, and dueDate
is a required field on PaymentFailedEmailData now rather than
optional — a reminder without it doesn't make sense.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/bulk-email-template.xlsx
+++ b/public/templates/bulk-email-template.xlsx
@@ -184,34 +184,28 @@
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
         <t>REQUIRED
-REQUIRED. Format YYYY-MM-DD, e.g. 2026-09-07. Cancellation date is auto-set to the next day.</t>
+REQUIRED. Format YYYY-MM-DD, e.g. 2026-09-14. Shown in the email as ‘Due date:’ — when this subscription is next charged. Cancellation date is auto-set to the day after.</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>REQUIRED
-REQUIRED. Format YYYY-MM-DD, e.g. 2026-09-14. Shown in the email as ‘Next due date:’ — when this subscription is next charged.</t>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <t>REQUIRED
 REQUIRED. Shown as ‘Affected subscriptions:’, e.g. QuickBooks Enterprise Silver Edition</t>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
+    <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <t>Optional
 Shown as ‘Payment method:’, e.g. VISA ending in 1234. Defaults to ‘the payment method on file’.</t>
       </text>
     </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
+    <comment ref="I1" authorId="0" shapeId="0">
       <text>
         <t>Optional
 Reference only — not shown in reminder emails.</t>
       </text>
     </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
+    <comment ref="J1" authorId="0" shapeId="0">
       <text>
         <t>Optional
 Reference only — not shown in reminder emails.</t>
@@ -510,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -519,11 +513,10 @@
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -554,30 +547,25 @@
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>Billing Date</t>
+          <t>Due Date</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>Due Date</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
           <t>Product</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Current Payment method</t>
+        </is>
+      </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Current Payment method</t>
+          <t>License Number</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>License Number</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>CAN</t>
         </is>
@@ -609,30 +597,25 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>QuickBooks Enterprise Silver Edition</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>QuickBooks Enterprise Silver Edition</t>
+          <t>VISA ending in 1234</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>VISA ending in 1234</t>
+          <t>1234-5678-9012-345</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>1234-5678-9012-345</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>CAN-00417</t>
         </is>

</xml_diff>

<commit_message>
Make Cancellation Date its own bulk column, not derived from Due Date
Cancellation Date was auto-computed as due date + 1 day. Now it's a
required column in the Excel template like Due Date, set directly by
whoever fills in the sheet rather than forced to always be the next
day. Same change on the client-side parser and validation.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/bulk-email-template.xlsx
+++ b/public/templates/bulk-email-template.xlsx
@@ -184,28 +184,34 @@
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
         <t>REQUIRED
-REQUIRED. Format YYYY-MM-DD, e.g. 2026-09-14. Shown in the email as ‘Due date:’ — when this subscription is next charged. Cancellation date is auto-set to the day after.</t>
+REQUIRED. Format YYYY-MM-DD, e.g. 2026-09-14. Shown in the email as ‘Due date:’ — when this subscription is next charged.</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>REQUIRED
+REQUIRED. Format YYYY-MM-DD, e.g. 2026-09-15. Shown in the email as ‘Cancellation date:’ — when the subscription cancels if payment isn’t fixed. Set this yourself; it is no longer auto-calculated.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <t>REQUIRED
 REQUIRED. Shown as ‘Affected subscriptions:’, e.g. QuickBooks Enterprise Silver Edition</t>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
+    <comment ref="I1" authorId="0" shapeId="0">
       <text>
         <t>Optional
 Shown as ‘Payment method:’, e.g. VISA ending in 1234. Defaults to ‘the payment method on file’.</t>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
+    <comment ref="J1" authorId="0" shapeId="0">
       <text>
         <t>Optional
 Reference only — not shown in reminder emails.</t>
       </text>
     </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
+    <comment ref="K1" authorId="0" shapeId="0">
       <text>
         <t>Optional
 Reference only — not shown in reminder emails.</t>
@@ -504,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -513,10 +519,11 @@
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -552,20 +559,25 @@
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
+          <t>Cancellation Date</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Current Payment method</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>License Number</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>CAN</t>
         </is>
@@ -602,20 +614,25 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
           <t>QuickBooks Enterprise Silver Edition</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>VISA ending in 1234</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>1234-5678-9012-345</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>CAN-00417</t>
         </is>

</xml_diff>

<commit_message>
Fix bulk email template's date format to match MM/DD/YYYY standard
The template's example dates and instruction comments told admins to use
YYYY-MM-DD, while the actual sent emails always rendered MM/DD/YYYY -- the
exact mismatch that caused confusion. Patched the underlying XML directly
(both cells and comment text) rather than rewriting through the xlsx
library, to preserve the sheet's styling and the Lists sheet's dropdown
validation untouched.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/bulk-email-template.xlsx
+++ b/public/templates/bulk-email-template.xlsx
@@ -185,13 +185,13 @@
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
         <t>REQUIRED
-REQUIRED. Format YYYY-MM-DD, e.g. 2026-09-14. Shown in the email as ‘Due date:’ — when this subscription is next charged.</t>
+REQUIRED. Format MM/DD/YYYY, e.g. 09/14/2026. Shown in the email as ‘Due date:’ — when this subscription is next charged.</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
         <t>REQUIRED
-REQUIRED. Format YYYY-MM-DD, e.g. 2026-09-15. Shown in the email as ‘Cancellation date:’ — when the subscription cancels if payment isn’t fixed. Set this yourself; it is no longer auto-calculated.</t>
+REQUIRED. Format MM/DD/YYYY, e.g. 09/15/2026. Shown in the email as ‘Cancellation date:’ — when the subscription cancels if payment isn’t fixed. Set this yourself; it is no longer auto-calculated.</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
@@ -610,12 +610,12 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>09/14/2026</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>09/15/2026</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">

</xml_diff>